<commit_message>
Updated logic to use Database
</commit_message>
<xml_diff>
--- a/New Records - Spools.xlsx
+++ b/New Records - Spools.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA17"/>
+  <dimension ref="A1:AA23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,50 +562,50 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>9991</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>93022</t>
+          <t>93170</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>424</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1-1</t>
+          <t>B-90991-12-1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1</t>
+          <t>B-90991-12</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02</t>
+          <t>B-90991</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>0</t>
@@ -613,17 +613,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>06CB1S02</t>
+          <t>W2JX</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -641,7 +641,7 @@
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -662,47 +662,47 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>30501--424</t>
+          <t>30511--2</t>
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>40472</v>
+        <v>40995</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>9992</v>
+        <v>5</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>93023</t>
+          <t>93174</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1-2</t>
+          <t>B-91041-1-1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1</t>
+          <t>B-91041-1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02</t>
+          <t>B-91041</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -722,17 +722,17 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>06CB1S02</t>
+          <t>EC57CAA</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -750,7 +750,7 @@
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>Weld Out</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -771,57 +771,57 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>30501--425</t>
+          <t>30511--6</t>
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>40473</v>
+        <v>40996</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>9993</v>
+        <v>6</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>93025</t>
+          <t>93175</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1-4</t>
+          <t>28105A-8-1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1</t>
+          <t>28105A-8</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02</t>
+          <t>28105A</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -831,17 +831,17 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>06CB1S02</t>
+          <t>3P1JX</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -859,7 +859,7 @@
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -880,47 +880,47 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>30501--427</t>
+          <t>30511--7</t>
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>40474</v>
+        <v>40997</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>9994</v>
+        <v>9</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>93026</t>
+          <t>93178</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>428</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1-5</t>
+          <t>28105B-1-2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02-1</t>
+          <t>28105B-1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1 1/2-BW3050010-06CB1S02</t>
+          <t>28105B</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -940,17 +940,17 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>06CB1S02</t>
+          <t>EC57CAA</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
@@ -968,7 +968,7 @@
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>Weld Out</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -989,79 +989,79 @@
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>30501--428</t>
+          <t>30511--10</t>
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>40475</v>
+        <v>40998</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>9995</v>
+        <v>17</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>93030</t>
+          <t>93186</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>432</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-1-1</t>
+          <t>28183-2-3</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-1</t>
+          <t>28183-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>28183</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>EC57CAA</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>01SA0U01</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>NONE</t>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R6" t="inlineStr"/>
@@ -1077,14 +1077,10 @@
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Cut</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>QC Complete</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
           <t>True</t>
@@ -1098,47 +1094,47 @@
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>30501--432</t>
+          <t>30511--18</t>
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>40476</v>
+        <v>40999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>9996</v>
+        <v>18</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>93031</t>
+          <t>93187</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>433</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-1-2</t>
+          <t>28184-1-1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-1</t>
+          <t>28184-1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>28184</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1148,7 +1144,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1158,7 +1154,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC55CAA</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,7 +1164,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1178,7 +1174,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>SEE NOTE</t>
         </is>
       </c>
       <c r="R7" t="inlineStr"/>
@@ -1186,7 +1182,7 @@
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
-          <t>QC</t>
+          <t>Cut</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1207,59 +1203,59 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>30501--433</t>
+          <t>30511--19</t>
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>40477</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>9997</v>
+        <v>24</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>93033</t>
+          <t>93193</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>435</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-1-4</t>
+          <t>28212-2-2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-1</t>
+          <t>28212-2</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>28212</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>0</t>
@@ -1267,7 +1263,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>3P1JX</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1277,7 +1273,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1287,7 +1283,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R8" t="inlineStr"/>
@@ -1295,7 +1291,7 @@
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1316,59 +1312,59 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>30501--435</t>
+          <t>30511--25</t>
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>40478</v>
+        <v>41001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>9998</v>
+        <v>26</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>93034</t>
+          <t>93195</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2-1</t>
+          <t>29970B-1-2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2</t>
+          <t>29970B-1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>29970B</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>0</t>
@@ -1376,7 +1372,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>W2JX</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1386,7 +1382,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1396,7 +1392,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R9" t="inlineStr"/>
@@ -1404,7 +1400,7 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1425,57 +1421,57 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>30501--436</t>
+          <t>30511--27</t>
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>40479</v>
+        <v>41002</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>9999</v>
+        <v>27</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>93035</t>
+          <t>93196</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>437</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2-2</t>
+          <t>B-91041-3-1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2</t>
+          <t>B-91041-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-91041</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1485,7 +1481,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC57CAA</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1495,7 +1491,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1505,7 +1501,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R10" t="inlineStr"/>
@@ -1513,7 +1509,7 @@
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>QC Complete</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1534,57 +1530,57 @@
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>30501--437</t>
+          <t>30511--28</t>
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>40480</v>
+        <v>41003</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>10000</v>
+        <v>28</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>93036</t>
+          <t>93197</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2-3</t>
+          <t>B-15729-1-1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2</t>
+          <t>B-15729-1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-15729</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1594,7 +1590,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC57CAA</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1604,7 +1600,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1614,7 +1610,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R11" t="inlineStr"/>
@@ -1622,7 +1618,7 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>Weld Out</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1643,47 +1639,47 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>30501--438</t>
+          <t>30511--29</t>
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>40481</v>
+        <v>41004</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>10001</v>
+        <v>29</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>93037</t>
+          <t>93198</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>439</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2-4</t>
+          <t>B-15729-2-1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-2</t>
+          <t>B-15729-2</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-15729</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1693,7 +1689,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1703,7 +1699,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC57CAA</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1713,7 +1709,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1723,7 +1719,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R12" t="inlineStr"/>
@@ -1731,7 +1727,7 @@
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>Weld Out</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1752,47 +1748,47 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>30501--439</t>
+          <t>30511--30</t>
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>40482</v>
+        <v>41005</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>10002</v>
+        <v>30</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>93038</t>
+          <t>93199</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3-1</t>
+          <t>B-15729-3-1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3</t>
+          <t>B-15729-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-15729</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1802,7 +1798,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1812,7 +1808,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC57CAA</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1822,7 +1818,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1832,7 +1828,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R13" t="inlineStr"/>
@@ -1840,7 +1836,7 @@
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1861,57 +1857,57 @@
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>30501--440</t>
+          <t>30511--31</t>
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>40483</v>
+        <v>41006</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>10003</v>
+        <v>31</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>93039</t>
+          <t>93200</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>441</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3-2</t>
+          <t>B-15729-4-1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3</t>
+          <t>B-15729-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-15729</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1921,7 +1917,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC57CAA</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1931,7 +1927,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1941,7 +1937,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R14" t="inlineStr"/>
@@ -1949,7 +1945,7 @@
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>QC Complete</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -1970,57 +1966,57 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>30501--441</t>
+          <t>30511--32</t>
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>40484</v>
+        <v>41007</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>10004</v>
+        <v>34</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>93040</t>
+          <t>93203</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>442</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3-3</t>
+          <t>B-15730-1-2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3</t>
+          <t>B-15730-1</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-15730</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2030,7 +2026,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC55CAA</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2040,7 +2036,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2050,7 +2046,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R15" t="inlineStr"/>
@@ -2058,7 +2054,7 @@
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -2079,57 +2075,57 @@
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>30501--442</t>
+          <t>30511--35</t>
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>40485</v>
+        <v>41008</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>10005</v>
+        <v>35</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>93041</t>
+          <t>93204</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>443</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3-4</t>
+          <t>B-15730-1-3</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3</t>
+          <t>B-15730-1</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-15730</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2139,7 +2135,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC55CAA</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2149,7 +2145,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2159,7 +2155,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R16" t="inlineStr"/>
@@ -2167,7 +2163,7 @@
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -2188,57 +2184,57 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>30501--443</t>
+          <t>30511--36</t>
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>40486</v>
+        <v>41009</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>10006</v>
+        <v>36</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>93042</t>
+          <t>93205</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>30501-</t>
+          <t>30511-</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3-5</t>
+          <t>B-15730-2-1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01-3</t>
+          <t>B-15730-2</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2-AI3050050-01SA0U01</t>
+          <t>B-15730</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2248,7 +2244,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>01SA0U01</t>
+          <t>EC55CAA</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2258,7 +2254,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2268,7 +2264,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>CFCS 6</t>
         </is>
       </c>
       <c r="R17" t="inlineStr"/>
@@ -2276,7 +2272,7 @@
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Cut</t>
+          <t>NDE</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2297,11 +2293,665 @@
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>30501--444</t>
+          <t>30511--37</t>
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>40487</v>
+        <v>41010</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>93206</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>30511-</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>B-15730-2-2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>B-15730-2</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>B-15730</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>EC55CAA</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>CFCS 6</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>QC Complete</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NDE Group is blank; </t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>30511--38</t>
+        </is>
+      </c>
+      <c r="AA18" t="n">
+        <v>41011</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>93207</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>30511-</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>B-15730-3-1</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>B-15730-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>B-15730</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>EC55CAA</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>CFCS 6</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>NDE</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NDE Group is blank; </t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>30511--39</t>
+        </is>
+      </c>
+      <c r="AA19" t="n">
+        <v>41012</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>93209</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>30511-</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>B-15730-4-1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>B-15730-4</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>B-15730</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>EC55CAA</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>SEE NOTE</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Final Fit</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NDE Group is blank; </t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>30511--41</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>41013</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>93211</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>30511-</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>B-15730-4-3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>B-15730-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>B-15730</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>EC55CAA</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>CFCS 6</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>QC Complete</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NDE Group is blank; </t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>30511--43</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>41014</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>93212</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>30511-</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>B-15730-4-4</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>B-15730-4</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>B-15730</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>EC55CAA</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>CFCS 6</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>QC Complete</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NDE Group is blank; </t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>30511--44</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>41015</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>93222</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>30511-</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>B-15729-3-2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>B-15729-3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>B-15729</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>EC57CAA</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>CFCS 6</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>QC Complete</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NDE Group is blank; </t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>30511--45</t>
+        </is>
+      </c>
+      <c r="AA23" t="n">
+        <v>41016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>